<commit_message>
excel file now shows the user who recorded the record
</commit_message>
<xml_diff>
--- a/bocfp-api/report/bocfp.xlsx
+++ b/bocfp-api/report/bocfp.xlsx
@@ -125,7 +125,19 @@
     <t>Date</t>
   </si>
   <si>
+    <t>User First Name</t>
+  </si>
+  <si>
+    <t>User Last Name</t>
+  </si>
+  <si>
     <t>Overweight</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Bocfp</t>
   </si>
   <si>
     <t>Underweight</t>
@@ -344,6 +356,8 @@
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -371,6 +385,12 @@
       <c r="H1" s="1" t="s">
         <v>36</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -389,13 +409,19 @@
         <v>79</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G2">
         <v>27.66009593501628</v>
       </c>
       <c r="H2" s="2">
         <v>44964.27569444444</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -415,13 +441,19 @@
         <v>59</v>
       </c>
       <c r="F3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G3">
         <v>29.260067446935132</v>
       </c>
       <c r="H3" s="2">
         <v>44963.68262731482</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -441,13 +473,19 @@
         <v>45</v>
       </c>
       <c r="F4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G4">
         <v>17.578125</v>
       </c>
       <c r="H4" s="2">
         <v>44963.582083333335</v>
+      </c>
+      <c r="I4" t="s">
+        <v>40</v>
+      </c>
+      <c r="J4" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -467,13 +505,19 @@
         <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G5">
         <v>19.47714681440443</v>
       </c>
       <c r="H5" s="2">
         <v>44961.76358796297</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6">
@@ -493,13 +537,19 @@
         <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G6">
         <v>15.967484395412978</v>
       </c>
       <c r="H6" s="2">
         <v>44961.76358796297</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
record now has soft delete
</commit_message>
<xml_diff>
--- a/bocfp-api/report/bocfp.xlsx
+++ b/bocfp-api/report/bocfp.xlsx
@@ -467,7 +467,7 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E4">
         <v>79</v>
@@ -479,7 +479,7 @@
         <v>27.66009593501628</v>
       </c>
       <c r="H4" s="2">
-        <v>44964.27569444444</v>
+        <v>44969.3205787037</v>
       </c>
       <c r="I4" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
date in the excel now formatting better
</commit_message>
<xml_diff>
--- a/bocfp-api/report/bocfp.xlsx
+++ b/bocfp-api/report/bocfp.xlsx
@@ -134,6 +134,9 @@
     <t>Overweight</t>
   </si>
   <si>
+    <t>Feb 07, 2023 12:22 AM</t>
+  </si>
+  <si>
     <t>Admin</t>
   </si>
   <si>
@@ -141,6 +144,15 @@
   </si>
   <si>
     <t>Underweight</t>
+  </si>
+  <si>
+    <t>Feb 06, 2023 09:58 PM</t>
+  </si>
+  <si>
+    <t>Feb 12, 2023 03:41 PM</t>
+  </si>
+  <si>
+    <t>Feb 05, 2023 02:19 AM</t>
   </si>
   <si>
     <t>Normal</t>
@@ -150,9 +162,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="100" formatCode="MMM DD, YYYY hh:mm AM/PM"/>
-  </numFmts>
   <fonts count="2">
     <font>
       <sz val="12"/>
@@ -186,10 +195,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf/>
     <xf fontId="1" applyFont="1"/>
-    <xf numFmtId="100" applyNumberFormat="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -414,14 +422,14 @@
       <c r="G2">
         <v>29.260067446935132</v>
       </c>
-      <c r="H2" s="2">
-        <v>44963.68262731482</v>
+      <c r="H2" t="s">
+        <v>40</v>
       </c>
       <c r="I2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -441,19 +449,19 @@
         <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G3">
         <v>17.578125</v>
       </c>
-      <c r="H3" s="2">
-        <v>44963.582083333335</v>
+      <c r="H3" t="s">
+        <v>44</v>
       </c>
       <c r="I3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -478,14 +486,14 @@
       <c r="G4">
         <v>27.66009593501628</v>
       </c>
-      <c r="H4" s="2">
-        <v>44969.3205787037</v>
+      <c r="H4" t="s">
+        <v>45</v>
       </c>
       <c r="I4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -505,19 +513,19 @@
         <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G5">
         <v>15.967484395412978</v>
       </c>
-      <c r="H5" s="2">
-        <v>44961.76358796297</v>
+      <c r="H5" t="s">
+        <v>46</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -537,19 +545,19 @@
         <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G6">
         <v>19.47714681440443</v>
       </c>
-      <c r="H6" s="2">
-        <v>44961.76358796297</v>
+      <c r="H6" t="s">
+        <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>